<commit_message>
A39 importer: grid section choice on the mapping screen, proposals of kept kinds only, tests
The mapping screen offers World events, Moments, or Chapters for a grid, with
start and stop labels for a band of rows and regions from row labels. Long
moment sheet headers guess to their fields. Claude's import proposals name
characters, moments, world events and open questions only (IM-5); the
recorded place proposal is now a moment. The fixture workbook gains a Hale
family moments sheet. Plot v1 Book Two chapters read after Book One.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/files/fixture-workbook.xlsx
+++ b/fixtures/files/fixture-workbook.xlsx
@@ -6,13 +6,14 @@
   <sheets>
     <sheet sheetId="1" name="People" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="High Level" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Hale family" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="75">
   <si>
     <t>ID</t>
   </si>
@@ -168,6 +169,75 @@
   </si>
   <si>
     <t>Pacific Rim accord</t>
+  </si>
+  <si>
+    <t>Chronological: Hale Family</t>
+  </si>
+  <si>
+    <t>POV</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>POV Age</t>
+  </si>
+  <si>
+    <t>Relevant World Events</t>
+  </si>
+  <si>
+    <t>How the POV Character Experiences This</t>
+  </si>
+  <si>
+    <t>Margaret meets Peter at the harbour</t>
+  </si>
+  <si>
+    <t>Margaret</t>
+  </si>
+  <si>
+    <t>A cold decade</t>
+  </si>
+  <si>
+    <t>Thinks he is too quiet</t>
+  </si>
+  <si>
+    <t>Peter and Margaret marry</t>
+  </si>
+  <si>
+    <t>Peter</t>
+  </si>
+  <si>
+    <t>Rain all spring</t>
+  </si>
+  <si>
+    <t>Nervous all day</t>
+  </si>
+  <si>
+    <t>Daniel is born</t>
+  </si>
+  <si>
+    <t>Satellite television arrives</t>
+  </si>
+  <si>
+    <t>Tired and proud</t>
+  </si>
+  <si>
+    <t>Meiling moves to Guangzhou</t>
+  </si>
+  <si>
+    <t>美玲</t>
+  </si>
+  <si>
+    <t>Guangdong opens to trade</t>
+  </si>
+  <si>
+    <t>Lonely the first year</t>
+  </si>
+  <si>
+    <t>Nobody remembers the storm</t>
+  </si>
+  <si>
+    <t>Ghost</t>
   </si>
 </sst>
 </file>
@@ -807,4 +877,126 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2">
+        <v>1980</v>
+      </c>
+      <c r="D2">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3">
+        <v>1982</v>
+      </c>
+      <c r="D3">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4">
+        <v>1985</v>
+      </c>
+      <c r="D4">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5">
+        <v>1990</v>
+      </c>
+      <c r="D5">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6">
+        <v>2001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
A39 importer: a people-by-year grid in the fixture workbook; e2e for moments by table and grid
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/files/fixture-workbook.xlsx
+++ b/fixtures/files/fixture-workbook.xlsx
@@ -7,13 +7,14 @@
     <sheet sheetId="1" name="People" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="High Level" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Hale family" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Lives by year" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
   <si>
     <t>ID</t>
   </si>
@@ -238,6 +239,15 @@
   </si>
   <si>
     <t>Ghost</t>
+  </si>
+  <si>
+    <t>Hale family</t>
+  </si>
+  <si>
+    <t>Moves to Portland</t>
+  </si>
+  <si>
+    <t>Starts school in Guangzhou</t>
   </si>
 </sst>
 </file>
@@ -999,4 +1009,50 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1">
+        <v>1980</v>
+      </c>
+      <c r="C1" s="1">
+        <v>1985</v>
+      </c>
+      <c r="D1" s="1">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
A39 importer review: real High Level A29 row, flag precedence row, family hints from sheet names and on the mapping screen
The integration suite runs the real High Level sheet: one Book One, four parts
of twelve chapters in sheet order, two strands each with one primary, the
Introduction in 2078, Siyuan primary in Part Four. Hand-made and renamed
chapters keep their newer values and file open questions. A sheet named for
families hints those families; the fixture moments sheet is now "Hale and Zhou
families". The mapping screen shows and edits the family hints.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/files/fixture-workbook.xlsx
+++ b/fixtures/files/fixture-workbook.xlsx
@@ -6,7 +6,7 @@
   <sheets>
     <sheet sheetId="1" name="People" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="High Level" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Hale family" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="Hale and Zhou families" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Lives by year" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -172,7 +172,7 @@
     <t>Pacific Rim accord</t>
   </si>
   <si>
-    <t>Chronological: Hale Family</t>
+    <t>Chronological: Hale and Zhou Families</t>
   </si>
   <si>
     <t>POV</t>

</xml_diff>